<commit_message>
Sync latest local files from CAMPS-Japan 8.12
Updates model, analysis, data/empirical, and outputs to match the
current local working copy (renamed model file, updated analysis
scripts, refreshed figures). data/validation large CSVs left
unchanged per current instructions.
</commit_message>
<xml_diff>
--- a/data/empirical/Japan 1994~2018 data collection.xlsx
+++ b/data/empirical/Japan 1994~2018 data collection.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonatachu/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sonatachu/Downloads/CAMPS-Japan/data/empirical/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04B5B163-7B03-A845-9D83-21D6592758C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AE76A1D-BADF-EA41-977A-C9ACC8E7AD38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15560" yWindow="660" windowWidth="19440" windowHeight="17580" activeTab="2" xr2:uid="{F55B0C82-C939-EC40-B15D-E340A69368EE}"/>
+    <workbookView xWindow="13860" yWindow="800" windowWidth="16380" windowHeight="16560" xr2:uid="{F55B0C82-C939-EC40-B15D-E340A69368EE}"/>
   </bookViews>
   <sheets>
     <sheet name="household age" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1635" uniqueCount="844">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1800" uniqueCount="891">
   <si>
     <t>Age</t>
   </si>
@@ -2585,6 +2585,489 @@
   </si>
   <si>
     <t>預金金利 3百万円 未満 / 1年 データコード IR02'DLDR43TL31Y</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>https://www.populationpyramid.net/india/1994/</t>
+  </si>
+  <si>
+    <t>comment：</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>https://www.populationpyramid.net/china/1994/</t>
+  </si>
+  <si>
+    <t>Finland</t>
+  </si>
+  <si>
+    <t>https://data.un.org/Data.aspx?d=POP&amp;f=tableCode%3A22%3BcountryCode%3A392</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>prob</t>
+  </si>
+  <si>
+    <t>9.7514.E-05</t>
+  </si>
+  <si>
+    <r>
+      <t>0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>20</t>
+    </r>
+  </si>
+  <si>
+    <t>1.2627.E-04</t>
+  </si>
+  <si>
+    <r>
+      <t>20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>40</t>
+    </r>
+  </si>
+  <si>
+    <t>1.3078.E-04</t>
+  </si>
+  <si>
+    <r>
+      <t>40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>60</t>
+    </r>
+  </si>
+  <si>
+    <t>1.5954.E-04</t>
+  </si>
+  <si>
+    <r>
+      <t>60</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>80</t>
+    </r>
+  </si>
+  <si>
+    <t>2.2483.E-04</t>
+  </si>
+  <si>
+    <r>
+      <t>80</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>100</t>
+    </r>
+  </si>
+  <si>
+    <t>3.5694.E-04</t>
+  </si>
+  <si>
+    <r>
+      <t>100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>120</t>
+    </r>
+  </si>
+  <si>
+    <t>5.8276.E-04</t>
+  </si>
+  <si>
+    <r>
+      <t>120</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>140</t>
+    </r>
+  </si>
+  <si>
+    <t>9.1400.E-04</t>
+  </si>
+  <si>
+    <r>
+      <t>140</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>160</t>
+    </r>
+  </si>
+  <si>
+    <t>1.4165.E-03</t>
+  </si>
+  <si>
+    <r>
+      <t>160</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>180</t>
+    </r>
+  </si>
+  <si>
+    <t>2.2473.E-03</t>
+  </si>
+  <si>
+    <r>
+      <t>180</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>200</t>
+    </r>
+  </si>
+  <si>
+    <t>3.4430.E-03</t>
+  </si>
+  <si>
+    <r>
+      <t>200</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>220</t>
+    </r>
+  </si>
+  <si>
+    <t>5.4644.E-03</t>
+  </si>
+  <si>
+    <r>
+      <t>220</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>240</t>
+    </r>
+  </si>
+  <si>
+    <t>9.5878.E-03</t>
+  </si>
+  <si>
+    <r>
+      <t>240</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>260</t>
+    </r>
+  </si>
+  <si>
+    <t>1.7547.E-02</t>
+  </si>
+  <si>
+    <r>
+      <t>260</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>280</t>
+    </r>
+  </si>
+  <si>
+    <t>3.0964.E-02</t>
+  </si>
+  <si>
+    <r>
+      <t>280</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>300</t>
+    </r>
+  </si>
+  <si>
+    <t>5.2730.E-02</t>
+  </si>
+  <si>
+    <r>
+      <t>300</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>320</t>
+    </r>
+  </si>
+  <si>
+    <t>8.3501.E-02</t>
+  </si>
+  <si>
+    <r>
+      <t>320</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>340</t>
+    </r>
+  </si>
+  <si>
+    <t>1.2674.E-01</t>
+  </si>
+  <si>
+    <r>
+      <t>340</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Hiragino Sans"/>
+      </rPr>
+      <t>～</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="2"/>
+      </rPr>
+      <t>360</t>
+    </r>
+  </si>
+  <si>
+    <t>ticks per year</t>
   </si>
 </sst>
 </file>
@@ -2603,7 +3086,7 @@
     <numFmt numFmtId="170" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="171" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="19">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2702,8 +3185,32 @@
       <color rgb="FF444444"/>
       <name val="Times"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Hiragino Sans"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2746,6 +3253,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2763,7 +3276,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -2853,6 +3366,20 @@
     <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="4" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="41" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
@@ -38179,16 +38706,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D9F4890-791D-474C-96A2-150691FB3097}">
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:AG42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="24">
+    <row r="1" spans="1:33" ht="24">
       <c r="A1" s="13" t="s">
         <v>202</v>
       </c>
@@ -38207,8 +38736,35 @@
       <c r="M1" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="2" spans="1:15">
+      <c r="Q1" s="13" t="s">
+        <v>844</v>
+      </c>
+      <c r="T1" t="s">
+        <v>207</v>
+      </c>
+      <c r="U1" t="s">
+        <v>63</v>
+      </c>
+      <c r="W1" s="13" t="s">
+        <v>848</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>207</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC1" s="13" t="s">
+        <v>850</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>207</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -38243,8 +38799,44 @@
       <c r="N2" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="3" spans="1:15">
+      <c r="Q2" t="s">
+        <v>0</v>
+      </c>
+      <c r="R2" t="s">
+        <v>1</v>
+      </c>
+      <c r="S2" t="s">
+        <v>62</v>
+      </c>
+      <c r="T2">
+        <v>500</v>
+      </c>
+      <c r="W2" t="s">
+        <v>0</v>
+      </c>
+      <c r="X2" t="s">
+        <v>1</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z2">
+        <v>500</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>62</v>
+      </c>
+      <c r="AF2">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33">
       <c r="A3" s="49">
         <v>5</v>
       </c>
@@ -38292,8 +38884,41 @@
         <v>256</v>
       </c>
       <c r="O3" s="3"/>
-    </row>
-    <row r="4" spans="1:15">
+      <c r="Q3" s="49" t="s">
+        <v>847</v>
+      </c>
+      <c r="S3" s="10"/>
+      <c r="U3">
+        <v>21</v>
+      </c>
+      <c r="W3" s="49">
+        <v>5</v>
+      </c>
+      <c r="X3" s="67"/>
+      <c r="Y3" s="7"/>
+      <c r="AA3">
+        <v>14</v>
+      </c>
+      <c r="AC3" s="49">
+        <v>5</v>
+      </c>
+      <c r="AD3" s="67">
+        <v>63941</v>
+      </c>
+      <c r="AE3" s="7">
+        <f>AD3/$AD$30</f>
+        <v>1.5531602941290778E-2</v>
+      </c>
+      <c r="AF3">
+        <f>AE3*$Z$2</f>
+        <v>7.7658014706453891</v>
+      </c>
+      <c r="AG3">
+        <f>ROUND(AF3,0)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:33">
       <c r="A4" s="49">
         <v>6</v>
       </c>
@@ -38301,7 +38926,7 @@
         <v>1302000</v>
       </c>
       <c r="C4" s="10">
-        <f t="shared" ref="C3:C28" si="5">B4/$B$30</f>
+        <f t="shared" ref="C4:C28" si="5">B4/$B$30</f>
         <v>1.2444920235899102E-2</v>
       </c>
       <c r="D4" s="11">
@@ -38341,8 +38966,40 @@
         <v>255</v>
       </c>
       <c r="O4" s="3"/>
-    </row>
-    <row r="5" spans="1:15">
+      <c r="Q4" s="49">
+        <v>6</v>
+      </c>
+      <c r="U4">
+        <v>21</v>
+      </c>
+      <c r="W4" s="49">
+        <v>6</v>
+      </c>
+      <c r="X4" s="67"/>
+      <c r="Y4" s="7"/>
+      <c r="AA4">
+        <v>14</v>
+      </c>
+      <c r="AC4" s="49">
+        <v>6</v>
+      </c>
+      <c r="AD4" s="67">
+        <v>62274</v>
+      </c>
+      <c r="AE4" s="7">
+        <f t="shared" ref="AE4:AE28" si="7">AD4/$AD$30</f>
+        <v>1.5126679932530645E-2</v>
+      </c>
+      <c r="AF4">
+        <f t="shared" ref="AF4:AF28" si="8">AE4*$Z$2</f>
+        <v>7.5633399662653229</v>
+      </c>
+      <c r="AG4">
+        <f t="shared" ref="AG4:AG28" si="9">ROUND(AF4,0)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:33">
       <c r="A5" s="49">
         <v>7</v>
       </c>
@@ -38390,8 +39047,40 @@
         <v>254</v>
       </c>
       <c r="O5" s="3"/>
-    </row>
-    <row r="6" spans="1:15">
+      <c r="Q5" s="49">
+        <v>7</v>
+      </c>
+      <c r="U5">
+        <v>20</v>
+      </c>
+      <c r="W5" s="49">
+        <v>7</v>
+      </c>
+      <c r="X5" s="67"/>
+      <c r="Y5" s="7"/>
+      <c r="AA5">
+        <v>14</v>
+      </c>
+      <c r="AC5" s="49">
+        <v>7</v>
+      </c>
+      <c r="AD5" s="67">
+        <v>61097</v>
+      </c>
+      <c r="AE5" s="7">
+        <f t="shared" si="7"/>
+        <v>1.4840780483634018E-2</v>
+      </c>
+      <c r="AF5">
+        <f t="shared" si="8"/>
+        <v>7.4203902418170093</v>
+      </c>
+      <c r="AG5">
+        <f t="shared" si="9"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:33">
       <c r="A6" s="49">
         <v>8</v>
       </c>
@@ -38439,8 +39128,40 @@
         <v>253</v>
       </c>
       <c r="O6" s="3"/>
-    </row>
-    <row r="7" spans="1:15">
+      <c r="Q6" s="49">
+        <v>8</v>
+      </c>
+      <c r="U6">
+        <v>20</v>
+      </c>
+      <c r="W6" s="49">
+        <v>8</v>
+      </c>
+      <c r="X6" s="67"/>
+      <c r="Y6" s="7"/>
+      <c r="AA6">
+        <v>14</v>
+      </c>
+      <c r="AC6" s="49">
+        <v>8</v>
+      </c>
+      <c r="AD6" s="67">
+        <v>62616</v>
+      </c>
+      <c r="AE6" s="7">
+        <f t="shared" si="7"/>
+        <v>1.5209753519210889E-2</v>
+      </c>
+      <c r="AF6">
+        <f t="shared" si="8"/>
+        <v>7.6048767596054443</v>
+      </c>
+      <c r="AG6">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:33">
       <c r="A7" s="49">
         <v>9</v>
       </c>
@@ -38488,8 +39209,40 @@
         <v>252</v>
       </c>
       <c r="O7" s="3"/>
-    </row>
-    <row r="8" spans="1:15">
+      <c r="Q7" s="49">
+        <v>9</v>
+      </c>
+      <c r="U7">
+        <v>19</v>
+      </c>
+      <c r="W7" s="49">
+        <v>9</v>
+      </c>
+      <c r="X7" s="67"/>
+      <c r="Y7" s="7"/>
+      <c r="AA7">
+        <v>14</v>
+      </c>
+      <c r="AC7" s="49">
+        <v>9</v>
+      </c>
+      <c r="AD7" s="67">
+        <v>64854</v>
+      </c>
+      <c r="AE7" s="7">
+        <f t="shared" si="7"/>
+        <v>1.575337541099564E-2</v>
+      </c>
+      <c r="AF7">
+        <f t="shared" si="8"/>
+        <v>7.8766877054978206</v>
+      </c>
+      <c r="AG7">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:33">
       <c r="A8" s="49">
         <v>10</v>
       </c>
@@ -38537,8 +39290,41 @@
         <v>251</v>
       </c>
       <c r="O8" s="3"/>
-    </row>
-    <row r="9" spans="1:15">
+      <c r="Q8" s="49">
+        <v>10</v>
+      </c>
+      <c r="S8" s="10"/>
+      <c r="U8">
+        <v>19</v>
+      </c>
+      <c r="W8" s="49">
+        <v>10</v>
+      </c>
+      <c r="X8" s="67"/>
+      <c r="Y8" s="7"/>
+      <c r="AA8">
+        <v>12</v>
+      </c>
+      <c r="AC8" s="49">
+        <v>10</v>
+      </c>
+      <c r="AD8" s="67">
+        <v>66940</v>
+      </c>
+      <c r="AE8" s="7">
+        <f t="shared" si="7"/>
+        <v>1.6260075708700281E-2</v>
+      </c>
+      <c r="AF8">
+        <f t="shared" si="8"/>
+        <v>8.1300378543501406</v>
+      </c>
+      <c r="AG8">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:33">
       <c r="A9" s="49">
         <v>11</v>
       </c>
@@ -38586,8 +39372,40 @@
         <v>250</v>
       </c>
       <c r="O9" s="3"/>
-    </row>
-    <row r="10" spans="1:15">
+      <c r="Q9" s="49">
+        <v>11</v>
+      </c>
+      <c r="U9">
+        <v>19</v>
+      </c>
+      <c r="W9" s="49">
+        <v>11</v>
+      </c>
+      <c r="X9" s="67"/>
+      <c r="Y9" s="7"/>
+      <c r="AA9">
+        <v>12</v>
+      </c>
+      <c r="AC9" s="49">
+        <v>11</v>
+      </c>
+      <c r="AD9" s="68">
+        <v>67583</v>
+      </c>
+      <c r="AE9" s="7">
+        <f t="shared" si="7"/>
+        <v>1.641626376786811E-2</v>
+      </c>
+      <c r="AF9">
+        <f t="shared" si="8"/>
+        <v>8.2081318839340547</v>
+      </c>
+      <c r="AG9">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:33">
       <c r="A10" s="49">
         <v>12</v>
       </c>
@@ -38635,8 +39453,40 @@
         <v>249</v>
       </c>
       <c r="O10" s="3"/>
-    </row>
-    <row r="11" spans="1:15">
+      <c r="Q10" s="49">
+        <v>12</v>
+      </c>
+      <c r="U10">
+        <v>18</v>
+      </c>
+      <c r="W10" s="49">
+        <v>12</v>
+      </c>
+      <c r="X10" s="67"/>
+      <c r="Y10" s="7"/>
+      <c r="AA10">
+        <v>12</v>
+      </c>
+      <c r="AC10" s="49">
+        <v>12</v>
+      </c>
+      <c r="AD10" s="67">
+        <v>66061</v>
+      </c>
+      <c r="AE10" s="7">
+        <f t="shared" si="7"/>
+        <v>1.6046562016618603E-2</v>
+      </c>
+      <c r="AF10">
+        <f t="shared" si="8"/>
+        <v>8.0232810083093007</v>
+      </c>
+      <c r="AG10">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:33">
       <c r="A11" s="49" t="s">
         <v>234</v>
       </c>
@@ -38684,8 +39534,40 @@
         <v>248</v>
       </c>
       <c r="O11" s="3"/>
-    </row>
-    <row r="12" spans="1:15">
+      <c r="Q11" s="49">
+        <v>13</v>
+      </c>
+      <c r="U11">
+        <v>18</v>
+      </c>
+      <c r="W11" s="49" t="s">
+        <v>234</v>
+      </c>
+      <c r="X11" s="67"/>
+      <c r="Y11" s="7"/>
+      <c r="AA11">
+        <v>12</v>
+      </c>
+      <c r="AC11" s="49" t="s">
+        <v>234</v>
+      </c>
+      <c r="AD11" s="67">
+        <v>64603</v>
+      </c>
+      <c r="AE11" s="7">
+        <f t="shared" si="7"/>
+        <v>1.5692406199718619E-2</v>
+      </c>
+      <c r="AF11">
+        <f t="shared" si="8"/>
+        <v>7.8462030998593093</v>
+      </c>
+      <c r="AG11">
+        <f>ROUND(AF11,0)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:33">
       <c r="A12" s="49" t="s">
         <v>233</v>
       </c>
@@ -38697,11 +39579,11 @@
         <v>1.5293296756865256E-2</v>
       </c>
       <c r="D12" s="11">
-        <f t="shared" ref="D12:D28" si="7">C12*$D$2</f>
+        <f t="shared" ref="D12:D28" si="10">C12*$D$2</f>
         <v>7.6466483784326282</v>
       </c>
       <c r="E12" s="52">
-        <f t="shared" ref="E12:E28" si="8">ROUND(D12,0)</f>
+        <f t="shared" ref="E12:E28" si="11">ROUND(D12,0)</f>
         <v>8</v>
       </c>
       <c r="F12" s="9" t="s">
@@ -38733,8 +39615,40 @@
         <v>247</v>
       </c>
       <c r="O12" s="3"/>
-    </row>
-    <row r="13" spans="1:15">
+      <c r="Q12" s="49">
+        <v>14</v>
+      </c>
+      <c r="U12">
+        <v>18</v>
+      </c>
+      <c r="W12" s="49" t="s">
+        <v>233</v>
+      </c>
+      <c r="X12" s="67"/>
+      <c r="Y12" s="7"/>
+      <c r="AA12">
+        <v>12</v>
+      </c>
+      <c r="AC12" s="49" t="s">
+        <v>233</v>
+      </c>
+      <c r="AD12" s="67">
+        <v>64445</v>
+      </c>
+      <c r="AE12" s="7">
+        <f t="shared" si="7"/>
+        <v>1.5654027174293244E-2</v>
+      </c>
+      <c r="AF12">
+        <f t="shared" si="8"/>
+        <v>7.827013587146622</v>
+      </c>
+      <c r="AG12">
+        <f t="shared" si="9"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:33">
       <c r="A13" s="28" t="s">
         <v>4</v>
       </c>
@@ -38782,8 +39696,62 @@
         <v>146</v>
       </c>
       <c r="O13" s="3"/>
-    </row>
-    <row r="14" spans="1:15">
+      <c r="Q13" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="R13" s="67">
+        <v>95235909</v>
+      </c>
+      <c r="S13" s="10">
+        <f>R13/$R$30</f>
+        <v>0.16225497662364852</v>
+      </c>
+      <c r="T13">
+        <f>S13*$T$2</f>
+        <v>81.127488311824266</v>
+      </c>
+      <c r="U13">
+        <f t="shared" ref="U13:U23" si="12">ROUND(T13,0)</f>
+        <v>81</v>
+      </c>
+      <c r="W13" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="X13" s="67">
+        <v>99213370</v>
+      </c>
+      <c r="Y13" s="7">
+        <f>X13/$X$30</f>
+        <v>0.11371426191806736</v>
+      </c>
+      <c r="Z13">
+        <f>Y13*$Z$2</f>
+        <v>56.857130959033675</v>
+      </c>
+      <c r="AA13">
+        <f>ROUND(Z13,0)</f>
+        <v>57</v>
+      </c>
+      <c r="AC13" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD13" s="67">
+        <v>326747</v>
+      </c>
+      <c r="AE13" s="7">
+        <f t="shared" si="7"/>
+        <v>7.9368553295349434E-2</v>
+      </c>
+      <c r="AF13">
+        <f>AE13*$AF$2</f>
+        <v>39.684276647674714</v>
+      </c>
+      <c r="AG13">
+        <f t="shared" si="9"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:33">
       <c r="A14" s="28" t="s">
         <v>5</v>
       </c>
@@ -38795,11 +39763,11 @@
         <v>9.5449288383785288E-2</v>
       </c>
       <c r="D14" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>47.724644191892644</v>
       </c>
       <c r="E14" s="29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>48</v>
       </c>
       <c r="F14" s="9" t="s">
@@ -38812,11 +39780,11 @@
         <v>6994000</v>
       </c>
       <c r="J14" s="7">
-        <f t="shared" ref="J14:J28" si="9">I14/$I$30</f>
+        <f t="shared" ref="J14:J28" si="13">I14/$I$30</f>
         <v>6.330271077521836E-2</v>
       </c>
       <c r="K14" s="31">
-        <f t="shared" ref="K14:K28" si="10">ROUND(J14*$K$2,3)</f>
+        <f t="shared" ref="K14:K28" si="14">ROUND(J14*$K$2,3)</f>
         <v>31.651</v>
       </c>
       <c r="L14" s="31">
@@ -38831,8 +39799,62 @@
         <v>147</v>
       </c>
       <c r="O14" s="3"/>
-    </row>
-    <row r="15" spans="1:15">
+      <c r="Q14" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="R14" s="67">
+        <v>84766745</v>
+      </c>
+      <c r="S14" s="10">
+        <f t="shared" ref="S13:S28" si="15">R14/$R$30</f>
+        <v>0.14441849059725753</v>
+      </c>
+      <c r="T14">
+        <f t="shared" ref="T13:T28" si="16">S14*$T$2</f>
+        <v>72.209245298628773</v>
+      </c>
+      <c r="U14">
+        <f t="shared" si="12"/>
+        <v>72</v>
+      </c>
+      <c r="W14" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="X14" s="67">
+        <v>127580296</v>
+      </c>
+      <c r="Y14" s="7">
+        <f t="shared" ref="Y14:Y28" si="17">X14/$X$30</f>
+        <v>0.14622725944022022</v>
+      </c>
+      <c r="Z14">
+        <f t="shared" ref="Z14:Z28" si="18">Y14*$Z$2</f>
+        <v>73.113629720110112</v>
+      </c>
+      <c r="AA14">
+        <f t="shared" ref="AA14:AA28" si="19">ROUND(Z14,0)</f>
+        <v>73</v>
+      </c>
+      <c r="AC14" s="28" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD14" s="67">
+        <v>304794</v>
+      </c>
+      <c r="AE14" s="7">
+        <f t="shared" si="7"/>
+        <v>7.4036054908240126E-2</v>
+      </c>
+      <c r="AF14">
+        <f t="shared" ref="AF14:AF28" si="20">AE14*$AF$2</f>
+        <v>37.018027454120066</v>
+      </c>
+      <c r="AG14">
+        <f t="shared" si="9"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:33">
       <c r="A15" s="32" t="s">
         <v>6</v>
       </c>
@@ -38844,11 +39866,11 @@
         <v>8.2899226732682726E-2</v>
       </c>
       <c r="D15" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>41.44961336634136</v>
       </c>
       <c r="E15" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>41</v>
       </c>
       <c r="F15" s="9" t="s">
@@ -38861,11 +39883,11 @@
         <v>7534000</v>
       </c>
       <c r="J15" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>6.8190252070416804E-2</v>
       </c>
       <c r="K15" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>34.094999999999999</v>
       </c>
       <c r="L15" s="31">
@@ -38880,8 +39902,62 @@
         <v>148</v>
       </c>
       <c r="O15" s="3"/>
-    </row>
-    <row r="16" spans="1:15">
+      <c r="Q15" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="R15" s="67">
+        <v>75168135</v>
+      </c>
+      <c r="S15" s="10">
+        <f t="shared" si="15"/>
+        <v>0.12806518166659442</v>
+      </c>
+      <c r="T15">
+        <f t="shared" si="16"/>
+        <v>64.032590833297206</v>
+      </c>
+      <c r="U15">
+        <f t="shared" si="12"/>
+        <v>64</v>
+      </c>
+      <c r="W15" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="X15" s="67">
+        <v>124897202</v>
+      </c>
+      <c r="Y15" s="7">
+        <f t="shared" si="17"/>
+        <v>0.14315200805155359</v>
+      </c>
+      <c r="Z15">
+        <f t="shared" si="18"/>
+        <v>71.576004025776797</v>
+      </c>
+      <c r="AA15">
+        <f t="shared" si="19"/>
+        <v>72</v>
+      </c>
+      <c r="AC15" s="32" t="s">
+        <v>6</v>
+      </c>
+      <c r="AD15" s="67">
+        <v>363105</v>
+      </c>
+      <c r="AE15" s="7">
+        <f t="shared" si="7"/>
+        <v>8.8200101437221637E-2</v>
+      </c>
+      <c r="AF15">
+        <f t="shared" si="20"/>
+        <v>44.100050718610817</v>
+      </c>
+      <c r="AG15">
+        <f t="shared" si="9"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:33">
       <c r="A16" s="32" t="s">
         <v>7</v>
       </c>
@@ -38893,11 +39969,11 @@
         <v>7.5481977805603076E-2</v>
       </c>
       <c r="D16" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>37.74098890280154</v>
       </c>
       <c r="E16" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>38</v>
       </c>
       <c r="F16" s="9" t="s">
@@ -38910,11 +39986,11 @@
         <v>8700000</v>
       </c>
       <c r="J16" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>7.8743720867086031E-2</v>
       </c>
       <c r="K16" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>39.372</v>
       </c>
       <c r="L16" s="31">
@@ -38929,8 +40005,62 @@
         <v>150</v>
       </c>
       <c r="O16" s="3"/>
-    </row>
-    <row r="17" spans="1:15">
+      <c r="Q16" s="32" t="s">
+        <v>7</v>
+      </c>
+      <c r="R16" s="67">
+        <v>67279771</v>
+      </c>
+      <c r="S16" s="10">
+        <f t="shared" si="15"/>
+        <v>0.11462564683295484</v>
+      </c>
+      <c r="T16">
+        <f t="shared" si="16"/>
+        <v>57.312823416477421</v>
+      </c>
+      <c r="U16">
+        <f t="shared" si="12"/>
+        <v>57</v>
+      </c>
+      <c r="W16" s="32" t="s">
+        <v>7</v>
+      </c>
+      <c r="X16" s="67">
+        <v>94608708</v>
+      </c>
+      <c r="Y16" s="7">
+        <f t="shared" si="17"/>
+        <v>0.10843658875050767</v>
+      </c>
+      <c r="Z16">
+        <f t="shared" si="18"/>
+        <v>54.218294375253834</v>
+      </c>
+      <c r="AA16">
+        <f t="shared" si="19"/>
+        <v>54</v>
+      </c>
+      <c r="AC16" s="32" t="s">
+        <v>7</v>
+      </c>
+      <c r="AD16" s="67">
+        <v>382159</v>
+      </c>
+      <c r="AE16" s="7">
+        <f t="shared" si="7"/>
+        <v>9.2828417579342556E-2</v>
+      </c>
+      <c r="AF16">
+        <f t="shared" si="20"/>
+        <v>46.414208789671278</v>
+      </c>
+      <c r="AG16">
+        <f t="shared" si="9"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:33">
       <c r="A17" s="32" t="s">
         <v>8</v>
       </c>
@@ -38942,11 +40072,11 @@
         <v>7.5568002599860448E-2</v>
       </c>
       <c r="D17" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>37.784001299930225</v>
       </c>
       <c r="E17" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>38</v>
       </c>
       <c r="F17" s="9" t="s">
@@ -38959,11 +40089,11 @@
         <v>9662000</v>
       </c>
       <c r="J17" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>8.7450785174458076E-2</v>
       </c>
       <c r="K17" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>43.725000000000001</v>
       </c>
       <c r="L17" s="31">
@@ -38978,8 +40108,61 @@
         <v>151</v>
       </c>
       <c r="O17" s="3"/>
-    </row>
-    <row r="18" spans="1:15">
+      <c r="Q17" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="R17" s="67">
+        <v>59185729</v>
+      </c>
+      <c r="S17" s="10">
+        <f t="shared" si="15"/>
+        <v>0.1008356950249574</v>
+      </c>
+      <c r="T17">
+        <f t="shared" si="16"/>
+        <v>50.417847512478701</v>
+      </c>
+      <c r="U17">
+        <f t="shared" si="12"/>
+        <v>50</v>
+      </c>
+      <c r="W17" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="X17" s="67">
+        <v>89480897</v>
+      </c>
+      <c r="Y17" s="7">
+        <f t="shared" si="17"/>
+        <v>0.10255930383295728</v>
+      </c>
+      <c r="Z17">
+        <f t="shared" si="18"/>
+        <v>51.279651916478642</v>
+      </c>
+      <c r="AA17">
+        <f t="shared" si="19"/>
+        <v>51</v>
+      </c>
+      <c r="AC17" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD17" s="67">
+        <v>391066</v>
+      </c>
+      <c r="AE17" s="7">
+        <f>AD17/$AD$30</f>
+        <v>9.4991974411392066E-2</v>
+      </c>
+      <c r="AF17">
+        <f t="shared" si="20"/>
+        <v>47.495987205696032</v>
+      </c>
+      <c r="AG17">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:33">
       <c r="A18" s="32" t="s">
         <v>9</v>
       </c>
@@ -38991,11 +40174,11 @@
         <v>9.074659963104921E-2</v>
       </c>
       <c r="D18" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>45.373299815524604</v>
       </c>
       <c r="E18" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>45</v>
       </c>
       <c r="F18" s="9" t="s">
@@ -39008,11 +40191,11 @@
         <v>8544000</v>
       </c>
       <c r="J18" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>7.7331764492917593E-2</v>
       </c>
       <c r="K18" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>38.665999999999997</v>
       </c>
       <c r="L18" s="31">
@@ -39027,8 +40210,61 @@
         <v>152</v>
       </c>
       <c r="O18" s="3"/>
-    </row>
-    <row r="19" spans="1:15">
+      <c r="Q18" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="R18" s="67">
+        <v>49587559</v>
+      </c>
+      <c r="S18" s="10">
+        <f t="shared" si="15"/>
+        <v>8.4483135729494549E-2</v>
+      </c>
+      <c r="T18">
+        <f t="shared" si="16"/>
+        <v>42.241567864747275</v>
+      </c>
+      <c r="U18">
+        <f t="shared" si="12"/>
+        <v>42</v>
+      </c>
+      <c r="W18" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="X18" s="67">
+        <v>82742216</v>
+      </c>
+      <c r="Y18" s="7">
+        <f t="shared" si="17"/>
+        <v>9.4835706335802364E-2</v>
+      </c>
+      <c r="Z18">
+        <f t="shared" si="18"/>
+        <v>47.417853167901185</v>
+      </c>
+      <c r="AA18">
+        <v>48</v>
+      </c>
+      <c r="AC18" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD18" s="67">
+        <v>413152</v>
+      </c>
+      <c r="AE18" s="7">
+        <f t="shared" si="7"/>
+        <v>0.10035677919332146</v>
+      </c>
+      <c r="AF18">
+        <f t="shared" si="20"/>
+        <v>50.178389596660729</v>
+      </c>
+      <c r="AG18">
+        <f>ROUND(AF18,0)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:33">
       <c r="A19" s="32" t="s">
         <v>10</v>
       </c>
@@ -39040,11 +40276,11 @@
         <v>9.5353705279054873E-2</v>
       </c>
       <c r="D19" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>47.676852639527439</v>
       </c>
       <c r="E19" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>48</v>
       </c>
       <c r="F19" s="9" t="s">
@@ -39057,11 +40293,11 @@
         <v>7779000</v>
       </c>
       <c r="J19" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>7.0407747658053133E-2</v>
       </c>
       <c r="K19" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>35.204000000000001</v>
       </c>
       <c r="L19" s="31">
@@ -39076,8 +40312,62 @@
         <v>153</v>
       </c>
       <c r="O19" s="3"/>
-    </row>
-    <row r="20" spans="1:15">
+      <c r="Q19" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="R19" s="67">
+        <v>36983471</v>
+      </c>
+      <c r="S19" s="10">
+        <f t="shared" si="15"/>
+        <v>6.3009344747960383E-2</v>
+      </c>
+      <c r="T19">
+        <f t="shared" si="16"/>
+        <v>31.504672373980192</v>
+      </c>
+      <c r="U19">
+        <f t="shared" si="12"/>
+        <v>32</v>
+      </c>
+      <c r="W19" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="X19" s="67">
+        <v>57717645</v>
+      </c>
+      <c r="Y19" s="7">
+        <f t="shared" si="17"/>
+        <v>6.6153577898059812E-2</v>
+      </c>
+      <c r="Z19">
+        <f t="shared" si="18"/>
+        <v>33.076788949029904</v>
+      </c>
+      <c r="AA19">
+        <f t="shared" si="19"/>
+        <v>33</v>
+      </c>
+      <c r="AC19" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD19" s="67">
+        <v>420464</v>
+      </c>
+      <c r="AE19" s="7">
+        <f t="shared" si="7"/>
+        <v>0.10213290219275405</v>
+      </c>
+      <c r="AF19">
+        <f t="shared" si="20"/>
+        <v>51.066451096377023</v>
+      </c>
+      <c r="AG19">
+        <f t="shared" si="9"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:33">
       <c r="A20" s="32" t="s">
         <v>11</v>
       </c>
@@ -39089,11 +40379,11 @@
         <v>8.6626967817168637E-2</v>
       </c>
       <c r="D20" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>43.313483908584317</v>
       </c>
       <c r="E20" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>43</v>
       </c>
       <c r="F20" s="9" t="s">
@@ -39106,11 +40396,11 @@
         <v>7774000</v>
       </c>
       <c r="J20" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>7.0362492646060551E-2</v>
       </c>
       <c r="K20" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>35.180999999999997</v>
       </c>
       <c r="L20" s="31">
@@ -39125,8 +40415,62 @@
         <v>154</v>
       </c>
       <c r="O20" s="3"/>
-    </row>
-    <row r="21" spans="1:15">
+      <c r="Q20" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="R20" s="67">
+        <v>30908896</v>
+      </c>
+      <c r="S20" s="10">
+        <f t="shared" si="15"/>
+        <v>5.2659991914843621E-2</v>
+      </c>
+      <c r="T20">
+        <f t="shared" si="16"/>
+        <v>26.329995957421811</v>
+      </c>
+      <c r="U20">
+        <f t="shared" si="12"/>
+        <v>26</v>
+      </c>
+      <c r="W20" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="X20" s="67">
+        <v>45807249</v>
+      </c>
+      <c r="Y20" s="7">
+        <f t="shared" si="17"/>
+        <v>5.2502374534119031E-2</v>
+      </c>
+      <c r="Z20">
+        <f t="shared" si="18"/>
+        <v>26.251187267059514</v>
+      </c>
+      <c r="AA20">
+        <f t="shared" si="19"/>
+        <v>26</v>
+      </c>
+      <c r="AC20" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD20" s="67">
+        <v>290788</v>
+      </c>
+      <c r="AE20" s="7">
+        <f t="shared" si="7"/>
+        <v>7.0633924337937526E-2</v>
+      </c>
+      <c r="AF20">
+        <f t="shared" si="20"/>
+        <v>35.316962168968765</v>
+      </c>
+      <c r="AG20">
+        <f t="shared" si="9"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:33">
       <c r="A21" s="32" t="s">
         <v>12</v>
       </c>
@@ -39138,11 +40482,11 @@
         <v>7.5061412144789286E-2</v>
       </c>
       <c r="D21" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>37.530706072394644</v>
       </c>
       <c r="E21" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>38</v>
       </c>
       <c r="F21" s="9" t="s">
@@ -39155,11 +40499,11 @@
         <v>9299000</v>
       </c>
       <c r="J21" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>8.416527130379689E-2</v>
       </c>
       <c r="K21" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>42.082999999999998</v>
       </c>
       <c r="L21" s="31">
@@ -39174,8 +40518,61 @@
         <v>155</v>
       </c>
       <c r="O21" s="3"/>
-    </row>
-    <row r="22" spans="1:15">
+      <c r="Q21" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="R21" s="67">
+        <v>27026379</v>
+      </c>
+      <c r="S21" s="10">
+        <f t="shared" si="15"/>
+        <v>4.6045284167622789E-2</v>
+      </c>
+      <c r="T21">
+        <f t="shared" si="16"/>
+        <v>23.022642083811395</v>
+      </c>
+      <c r="U21">
+        <f t="shared" si="12"/>
+        <v>23</v>
+      </c>
+      <c r="W21" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="X21" s="67">
+        <v>42593611</v>
+      </c>
+      <c r="Y21" s="7">
+        <f t="shared" si="17"/>
+        <v>4.8819035552267555E-2</v>
+      </c>
+      <c r="Z21">
+        <f t="shared" si="18"/>
+        <v>24.409517776133779</v>
+      </c>
+      <c r="AA21">
+        <v>25</v>
+      </c>
+      <c r="AC21" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="AD21" s="67">
+        <v>266433</v>
+      </c>
+      <c r="AE21" s="7">
+        <f t="shared" si="7"/>
+        <v>6.4717967602272816E-2</v>
+      </c>
+      <c r="AF21">
+        <f t="shared" si="20"/>
+        <v>32.358983801136411</v>
+      </c>
+      <c r="AG21">
+        <f t="shared" si="9"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:33">
       <c r="A22" s="32" t="s">
         <v>13</v>
       </c>
@@ -39187,11 +40584,11 @@
         <v>6.9957274352185503E-2</v>
       </c>
       <c r="D22" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>34.978637176092754</v>
       </c>
       <c r="E22" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>35</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -39204,11 +40601,11 @@
         <v>9260000</v>
       </c>
       <c r="J22" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>8.3812282210254788E-2</v>
       </c>
       <c r="K22" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>41.905999999999999</v>
       </c>
       <c r="L22" s="31">
@@ -39223,8 +40620,62 @@
         <v>156</v>
       </c>
       <c r="O22" s="3"/>
-    </row>
-    <row r="23" spans="1:15">
+      <c r="Q22" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="R22" s="67">
+        <v>21787139</v>
+      </c>
+      <c r="S22" s="10">
+        <f t="shared" si="15"/>
+        <v>3.7119105243602818E-2</v>
+      </c>
+      <c r="T22">
+        <f t="shared" si="16"/>
+        <v>18.559552621801409</v>
+      </c>
+      <c r="U22">
+        <f t="shared" si="12"/>
+        <v>19</v>
+      </c>
+      <c r="W22" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="X22" s="67">
+        <v>36684518</v>
+      </c>
+      <c r="Y22" s="7">
+        <f t="shared" si="17"/>
+        <v>4.2046277514714563E-2</v>
+      </c>
+      <c r="Z22">
+        <f t="shared" si="18"/>
+        <v>21.02313875735728</v>
+      </c>
+      <c r="AA22">
+        <f t="shared" si="19"/>
+        <v>21</v>
+      </c>
+      <c r="AC22" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="AD22" s="67">
+        <v>245204</v>
+      </c>
+      <c r="AE22" s="7">
+        <f t="shared" si="7"/>
+        <v>5.9561332597492439E-2</v>
+      </c>
+      <c r="AF22">
+        <f t="shared" si="20"/>
+        <v>29.780666298746219</v>
+      </c>
+      <c r="AG22">
+        <f t="shared" si="9"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:33">
       <c r="A23" s="34" t="s">
         <v>14</v>
       </c>
@@ -39236,11 +40687,11 @@
         <v>5.9529157626098013E-2</v>
       </c>
       <c r="D23" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>29.764578813049006</v>
       </c>
       <c r="E23" s="37">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>30</v>
       </c>
       <c r="F23" s="9" t="s">
@@ -39253,11 +40704,11 @@
         <v>8334000</v>
       </c>
       <c r="J23" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>7.5431053989229307E-2</v>
       </c>
       <c r="K23" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>37.716000000000001</v>
       </c>
       <c r="L23" s="31">
@@ -39272,8 +40723,62 @@
         <v>157</v>
       </c>
       <c r="O23" s="3"/>
-    </row>
-    <row r="24" spans="1:15">
+      <c r="Q23" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="R23" s="67">
+        <v>16248705</v>
+      </c>
+      <c r="S23" s="10">
+        <f t="shared" si="15"/>
+        <v>2.7683184605709604E-2</v>
+      </c>
+      <c r="T23">
+        <f t="shared" si="16"/>
+        <v>13.841592302854801</v>
+      </c>
+      <c r="U23">
+        <f t="shared" si="12"/>
+        <v>14</v>
+      </c>
+      <c r="W23" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="X23" s="67">
+        <v>28336243</v>
+      </c>
+      <c r="Y23" s="7">
+        <f t="shared" si="17"/>
+        <v>3.247782993638864E-2</v>
+      </c>
+      <c r="Z23">
+        <f t="shared" si="18"/>
+        <v>16.238914968194319</v>
+      </c>
+      <c r="AA23">
+        <f t="shared" si="19"/>
+        <v>16</v>
+      </c>
+      <c r="AC23" s="34" t="s">
+        <v>14</v>
+      </c>
+      <c r="AD23" s="67">
+        <v>232011</v>
+      </c>
+      <c r="AE23" s="7">
+        <f>AD23/$AD$30</f>
+        <v>5.6356683974473576E-2</v>
+      </c>
+      <c r="AF23">
+        <f t="shared" si="20"/>
+        <v>28.178341987236788</v>
+      </c>
+      <c r="AG23">
+        <f t="shared" si="9"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:33">
       <c r="A24" s="34" t="s">
         <v>15</v>
       </c>
@@ -39285,11 +40790,11 @@
         <v>4.2926372334426165E-2</v>
       </c>
       <c r="D24" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>21.463186167213081</v>
       </c>
       <c r="E24" s="37">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>21</v>
       </c>
       <c r="F24" s="9" t="s">
@@ -39302,11 +40807,11 @@
         <v>6905000</v>
       </c>
       <c r="J24" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>6.2497171561750463E-2</v>
       </c>
       <c r="K24" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>31.248999999999999</v>
       </c>
       <c r="L24" s="31">
@@ -39321,8 +40826,61 @@
         <v>158</v>
       </c>
       <c r="O24" s="3"/>
-    </row>
-    <row r="25" spans="1:15">
+      <c r="Q24" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="R24" s="67">
+        <v>11056270</v>
+      </c>
+      <c r="S24" s="10">
+        <f t="shared" si="15"/>
+        <v>1.8836748126116444E-2</v>
+      </c>
+      <c r="T24">
+        <f t="shared" si="16"/>
+        <v>9.4183740630582218</v>
+      </c>
+      <c r="U24">
+        <v>10</v>
+      </c>
+      <c r="W24" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="X24" s="67">
+        <v>20433376</v>
+      </c>
+      <c r="Y24" s="7">
+        <f t="shared" si="17"/>
+        <v>2.3419890588681259E-2</v>
+      </c>
+      <c r="Z24">
+        <f t="shared" si="18"/>
+        <v>11.709945294340629</v>
+      </c>
+      <c r="AA24">
+        <f t="shared" si="19"/>
+        <v>12</v>
+      </c>
+      <c r="AC24" s="34" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD24" s="67">
+        <v>188813</v>
+      </c>
+      <c r="AE24" s="7">
+        <f t="shared" si="7"/>
+        <v>4.5863664098996511E-2</v>
+      </c>
+      <c r="AF24">
+        <f t="shared" si="20"/>
+        <v>22.931832049498254</v>
+      </c>
+      <c r="AG24">
+        <f t="shared" si="9"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:33">
       <c r="A25" s="34" t="s">
         <v>16</v>
       </c>
@@ -39334,11 +40892,11 @@
         <v>3.0080003058659353E-2</v>
       </c>
       <c r="D25" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>15.040001529329677</v>
       </c>
       <c r="E25" s="37">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>15</v>
       </c>
       <c r="F25" s="9" t="s">
@@ -39351,11 +40909,11 @@
         <v>5783000</v>
       </c>
       <c r="J25" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>5.234194687061592E-2</v>
       </c>
       <c r="K25" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>26.170999999999999</v>
       </c>
       <c r="L25" s="31">
@@ -39370,8 +40928,62 @@
         <v>159</v>
       </c>
       <c r="O25" s="3"/>
-    </row>
-    <row r="26" spans="1:15">
+      <c r="Q25" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="R25" s="67">
+        <v>6672529</v>
+      </c>
+      <c r="S25" s="10">
+        <f t="shared" si="15"/>
+        <v>1.1368096847961169E-2</v>
+      </c>
+      <c r="T25">
+        <f t="shared" si="16"/>
+        <v>5.6840484239805846</v>
+      </c>
+      <c r="U25">
+        <f>ROUND(T25,0)</f>
+        <v>6</v>
+      </c>
+      <c r="W25" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="X25" s="67">
+        <v>12813324</v>
+      </c>
+      <c r="Y25" s="7">
+        <f t="shared" si="17"/>
+        <v>1.4686102098709665E-2</v>
+      </c>
+      <c r="Z25">
+        <f t="shared" si="18"/>
+        <v>7.3430510493548322</v>
+      </c>
+      <c r="AA25">
+        <f t="shared" si="19"/>
+        <v>7</v>
+      </c>
+      <c r="AC25" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="AD25" s="67">
+        <v>132603</v>
+      </c>
+      <c r="AE25" s="7">
+        <f t="shared" si="7"/>
+        <v>3.2209961446082812E-2</v>
+      </c>
+      <c r="AF25">
+        <f>AE25*$AF$2</f>
+        <v>16.104980723041407</v>
+      </c>
+      <c r="AG25">
+        <f t="shared" si="9"/>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:33">
       <c r="A26" s="34" t="s">
         <v>17</v>
       </c>
@@ -39383,11 +40995,11 @@
         <v>2.1458407011976564E-2</v>
       </c>
       <c r="D26" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>10.729203505988282</v>
       </c>
       <c r="E26" s="37">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>11</v>
       </c>
       <c r="F26" s="9" t="s">
@@ -39400,11 +41012,11 @@
         <v>4202000</v>
       </c>
       <c r="J26" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>3.8032312078562704E-2</v>
       </c>
       <c r="K26" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>19.015999999999998</v>
       </c>
       <c r="L26" s="31">
@@ -39419,8 +41031,62 @@
         <v>160</v>
       </c>
       <c r="O26" s="3"/>
-    </row>
-    <row r="27" spans="1:15">
+      <c r="Q26" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="R26" s="67">
+        <v>3337654</v>
+      </c>
+      <c r="S26" s="10">
+        <f t="shared" si="15"/>
+        <v>5.6864157378686535E-3</v>
+      </c>
+      <c r="T26">
+        <f t="shared" si="16"/>
+        <v>2.8432078689343268</v>
+      </c>
+      <c r="U26">
+        <f>ROUND(T26,0)</f>
+        <v>3</v>
+      </c>
+      <c r="W26" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="X26" s="67">
+        <v>6541768</v>
+      </c>
+      <c r="Y26" s="7">
+        <f t="shared" si="17"/>
+        <v>7.4979039595090028E-3</v>
+      </c>
+      <c r="Z26">
+        <f t="shared" si="18"/>
+        <v>3.7489519797545015</v>
+      </c>
+      <c r="AA26">
+        <f t="shared" si="19"/>
+        <v>4</v>
+      </c>
+      <c r="AC26" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD26" s="67">
+        <v>97364</v>
+      </c>
+      <c r="AE26" s="7">
+        <f t="shared" si="7"/>
+        <v>2.3650224250102991E-2</v>
+      </c>
+      <c r="AF26">
+        <f t="shared" si="20"/>
+        <v>11.825112125051495</v>
+      </c>
+      <c r="AG26">
+        <f t="shared" si="9"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:33">
       <c r="A27" s="34" t="s">
         <v>18</v>
       </c>
@@ -39432,11 +41098,11 @@
         <v>1.009357585953107E-2</v>
       </c>
       <c r="D27" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>5.0467879297655349</v>
       </c>
       <c r="E27" s="37">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="F27" s="9" t="s">
@@ -39449,11 +41115,11 @@
         <v>2332000</v>
       </c>
       <c r="J27" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>2.1106937593338461E-2</v>
       </c>
       <c r="K27" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>10.553000000000001</v>
       </c>
       <c r="L27" s="31">
@@ -39468,8 +41134,62 @@
         <v>161</v>
       </c>
       <c r="O27" s="3"/>
-    </row>
-    <row r="28" spans="1:15">
+      <c r="Q27" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="R27" s="67">
+        <v>1304761</v>
+      </c>
+      <c r="S27" s="10">
+        <f t="shared" si="15"/>
+        <v>2.2229426670821008E-3</v>
+      </c>
+      <c r="T27">
+        <f t="shared" si="16"/>
+        <v>1.1114713335410504</v>
+      </c>
+      <c r="U27">
+        <f>ROUND(T27,0)</f>
+        <v>1</v>
+      </c>
+      <c r="W27" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="X27" s="67">
+        <v>2413648</v>
+      </c>
+      <c r="Y27" s="7">
+        <f t="shared" si="17"/>
+        <v>2.766423525881839E-3</v>
+      </c>
+      <c r="Z27">
+        <f t="shared" si="18"/>
+        <v>1.3832117629409195</v>
+      </c>
+      <c r="AA27">
+        <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="AC27" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD27" s="67">
+        <v>46398</v>
+      </c>
+      <c r="AE27" s="7">
+        <f t="shared" si="7"/>
+        <v>1.1270316592953028E-2</v>
+      </c>
+      <c r="AF27">
+        <f t="shared" si="20"/>
+        <v>5.6351582964765141</v>
+      </c>
+      <c r="AG27">
+        <f t="shared" si="9"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:33">
       <c r="A28" s="34" t="s">
         <v>235</v>
       </c>
@@ -39481,11 +41201,11 @@
         <v>4.0049320882040891E-3</v>
       </c>
       <c r="D28" s="11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>2.0024660441020448</v>
       </c>
       <c r="E28" s="37">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>2</v>
       </c>
       <c r="F28" s="9" t="s">
@@ -39498,11 +41218,11 @@
         <v>1290000</v>
       </c>
       <c r="J28" s="7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="13"/>
         <v>1.167579309408517E-2</v>
       </c>
       <c r="K28" s="31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="14"/>
         <v>5.8380000000000001</v>
       </c>
       <c r="L28" s="31">
@@ -39517,12 +41237,68 @@
         <v>162</v>
       </c>
       <c r="O28" s="3"/>
-    </row>
-    <row r="29" spans="1:15">
+      <c r="Q28" s="34" t="s">
+        <v>235</v>
+      </c>
+      <c r="R28" s="67">
+        <v>402508</v>
+      </c>
+      <c r="S28" s="10">
+        <f t="shared" si="15"/>
+        <v>6.8575946632516011E-4</v>
+      </c>
+      <c r="T28">
+        <f t="shared" si="16"/>
+        <v>0.34287973316258002</v>
+      </c>
+      <c r="U28">
+        <f>ROUND(T28,0)</f>
+        <v>0</v>
+      </c>
+      <c r="W28" s="34" t="s">
+        <v>235</v>
+      </c>
+      <c r="X28" s="67">
+        <v>615496</v>
+      </c>
+      <c r="Y28" s="7">
+        <f t="shared" si="17"/>
+        <v>7.054560625601447E-4</v>
+      </c>
+      <c r="Z28">
+        <f t="shared" si="18"/>
+        <v>0.35272803128007235</v>
+      </c>
+      <c r="AA28">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="AC28" s="34" t="s">
+        <v>235</v>
+      </c>
+      <c r="AD28" s="67">
+        <f>15550+181</f>
+        <v>15731</v>
+      </c>
+      <c r="AE28" s="7">
+        <f t="shared" si="7"/>
+        <v>3.8211420820669873E-3</v>
+      </c>
+      <c r="AF28">
+        <f t="shared" si="20"/>
+        <v>1.9105710410334937</v>
+      </c>
+      <c r="AG28">
+        <f t="shared" si="9"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:33">
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
-    </row>
-    <row r="30" spans="1:15">
+      <c r="R29" s="67"/>
+    </row>
+    <row r="30" spans="1:33">
       <c r="A30" s="34" t="s">
         <v>236</v>
       </c>
@@ -39556,40 +41332,195 @@
         <v>527</v>
       </c>
       <c r="O30" s="3"/>
-    </row>
-    <row r="31" spans="1:15">
+      <c r="Q30" s="34" t="s">
+        <v>236</v>
+      </c>
+      <c r="R30" s="3">
+        <f>SUM(R13:R28)</f>
+        <v>586952160</v>
+      </c>
+      <c r="W30" s="34" t="s">
+        <v>236</v>
+      </c>
+      <c r="X30" s="67">
+        <f>SUM(X13:X28)</f>
+        <v>872479567</v>
+      </c>
+      <c r="AA30">
+        <f>SUM(AA13:AA28)</f>
+        <v>500</v>
+      </c>
+      <c r="AC30" s="34" t="s">
+        <v>236</v>
+      </c>
+      <c r="AD30" s="67">
+        <f>SUM(AD13:AD28)</f>
+        <v>4116832</v>
+      </c>
+      <c r="AG30">
+        <f>SUM(AG13:AG28)</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="31" spans="1:33">
       <c r="F31">
         <f>SUM(E23:E28)/SUM(E13:E22)</f>
         <v>0.20192307692307693</v>
       </c>
-    </row>
-    <row r="32" spans="1:15">
+      <c r="Q31" s="67"/>
+      <c r="S31" s="12"/>
+    </row>
+    <row r="32" spans="1:33">
       <c r="D32" s="3">
         <f>SUM(B4:B12)</f>
         <v>13109000</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:33">
       <c r="C34" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="35" spans="1:3">
+      <c r="Q34" t="s">
+        <v>845</v>
+      </c>
+      <c r="W34" t="s">
+        <v>849</v>
+      </c>
+      <c r="AC34" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="35" spans="1:33">
       <c r="C35" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="37" spans="1:33">
+      <c r="Q37" t="s">
+        <v>846</v>
+      </c>
+      <c r="W37" t="s">
+        <v>846</v>
+      </c>
+      <c r="AC37" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="38" spans="1:33">
       <c r="A38" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="41" spans="1:3">
+      <c r="Q38" s="69" t="s">
+        <v>2</v>
+      </c>
+      <c r="R38" s="70">
+        <v>118917525</v>
+      </c>
+      <c r="S38" s="71">
+        <v>0.2026</v>
+      </c>
+      <c r="T38" s="72">
+        <v>101.300867</v>
+      </c>
+      <c r="U38" s="72">
+        <v>101</v>
+      </c>
+      <c r="W38" s="69" t="s">
+        <v>2</v>
+      </c>
+      <c r="X38" s="73">
+        <v>121762077</v>
+      </c>
+      <c r="Y38" s="7">
+        <f>X38/X30</f>
+        <v>0.13955865742354973</v>
+      </c>
+      <c r="Z38">
+        <f>Z2*Y38</f>
+        <v>69.779328711774866</v>
+      </c>
+      <c r="AA38">
+        <f>ROUND(Z38,0)</f>
+        <v>70</v>
+      </c>
+      <c r="AC38" s="69" t="s">
+        <v>2</v>
+      </c>
+      <c r="AD38">
+        <v>314781</v>
+      </c>
+      <c r="AE38" s="7">
+        <f>AD38/AD30</f>
+        <v>7.6461949382437763E-2</v>
+      </c>
+      <c r="AF38">
+        <f>AE38*AF2</f>
+        <v>38.230974691218883</v>
+      </c>
+      <c r="AG38">
+        <f>ROUND(AF38,0)</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:33">
+      <c r="Q39" s="69" t="s">
+        <v>3</v>
+      </c>
+      <c r="R39" s="70">
+        <v>107695663</v>
+      </c>
+      <c r="S39" s="71">
+        <v>0.1835</v>
+      </c>
+      <c r="T39" s="72">
+        <v>91.741431700000007</v>
+      </c>
+      <c r="U39" s="72">
+        <v>92</v>
+      </c>
+      <c r="W39" s="69" t="s">
+        <v>3</v>
+      </c>
+      <c r="X39" s="73">
+        <v>104531206</v>
+      </c>
+      <c r="Y39" s="7">
+        <f>X39/X30</f>
+        <v>0.11980934563250351</v>
+      </c>
+      <c r="Z39">
+        <f>Z2*Y39</f>
+        <v>59.904672816251754</v>
+      </c>
+      <c r="AA39">
+        <f>ROUND(Z39,0)</f>
+        <v>60</v>
+      </c>
+      <c r="AC39" s="69" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD39">
+        <v>329639</v>
+      </c>
+      <c r="AE39" s="7">
+        <f>AD39/AD30</f>
+        <v>8.0071035203768334E-2</v>
+      </c>
+      <c r="AF39">
+        <f>AE39*AF2</f>
+        <v>40.035517601884166</v>
+      </c>
+      <c r="AG39">
+        <f>ROUND(AF39,0)</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:33">
       <c r="A41" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:33">
       <c r="A42" s="14" t="s">
         <v>258</v>
       </c>
@@ -39599,6 +41530,7 @@
     <hyperlink ref="A42" r:id="rId1" xr:uid="{2FEC7821-3CC7-8146-B0BB-CCEE4103580F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
@@ -47417,13 +49349,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE25E9BC-486D-8D49-BA27-774F50E684A7}">
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:W27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16"/>
   <cols>
     <col min="6" max="7" width="12.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
+    <row r="1" spans="1:23">
       <c r="E1">
         <v>4</v>
       </c>
@@ -47448,8 +49380,11 @@
       <c r="Q1" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="3" spans="1:17">
+      <c r="S1" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -47498,8 +49433,23 @@
       <c r="Q3" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" ht="17">
+      <c r="S3" s="74" t="s">
+        <v>223</v>
+      </c>
+      <c r="T3" s="74" t="s">
+        <v>852</v>
+      </c>
+      <c r="U3" s="74" t="s">
+        <v>853</v>
+      </c>
+      <c r="V3" s="74" t="s">
+        <v>168</v>
+      </c>
+      <c r="W3" s="74" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" ht="17">
       <c r="A4" t="s">
         <v>53</v>
       </c>
@@ -47542,8 +49492,23 @@
       </c>
       <c r="P4" s="10"/>
       <c r="Q4" s="9"/>
-    </row>
-    <row r="5" spans="1:17" ht="17">
+      <c r="S4" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T4" s="75" t="s">
+        <v>4</v>
+      </c>
+      <c r="U4" s="75">
+        <v>3.8999999999999999E-4</v>
+      </c>
+      <c r="V4" s="75" t="s">
+        <v>854</v>
+      </c>
+      <c r="W4" s="75" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" ht="17">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -47586,8 +49551,23 @@
       </c>
       <c r="P5" s="10"/>
       <c r="Q5" s="9"/>
-    </row>
-    <row r="6" spans="1:17" ht="17">
+      <c r="S5" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T5" s="75" t="s">
+        <v>5</v>
+      </c>
+      <c r="U5" s="75">
+        <v>5.0500000000000002E-4</v>
+      </c>
+      <c r="V5" s="75" t="s">
+        <v>856</v>
+      </c>
+      <c r="W5" s="75" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" ht="17">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -47630,8 +49610,23 @@
       </c>
       <c r="P6" s="10"/>
       <c r="Q6" s="9"/>
-    </row>
-    <row r="7" spans="1:17" ht="17">
+      <c r="S6" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T6" s="75" t="s">
+        <v>6</v>
+      </c>
+      <c r="U6" s="75">
+        <v>5.2300000000000003E-4</v>
+      </c>
+      <c r="V6" s="75" t="s">
+        <v>858</v>
+      </c>
+      <c r="W6" s="75" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="17">
       <c r="A7" t="s">
         <v>53</v>
       </c>
@@ -47672,8 +49667,23 @@
         <v>8.8999999999999995E-5</v>
       </c>
       <c r="P7" s="10"/>
-    </row>
-    <row r="8" spans="1:17" ht="17">
+      <c r="S7" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T7" s="75" t="s">
+        <v>7</v>
+      </c>
+      <c r="U7" s="75">
+        <v>6.38E-4</v>
+      </c>
+      <c r="V7" s="75" t="s">
+        <v>860</v>
+      </c>
+      <c r="W7" s="75" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" ht="17">
       <c r="A8" t="s">
         <v>53</v>
       </c>
@@ -47726,8 +49736,23 @@
       <c r="Q8" s="9" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="17">
+      <c r="S8" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T8" s="75" t="s">
+        <v>8</v>
+      </c>
+      <c r="U8" s="75">
+        <v>8.9899999999999995E-4</v>
+      </c>
+      <c r="V8" s="75" t="s">
+        <v>862</v>
+      </c>
+      <c r="W8" s="75" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="17">
       <c r="A9" t="s">
         <v>53</v>
       </c>
@@ -47780,8 +49805,23 @@
       <c r="Q9" s="9" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" ht="17">
+      <c r="S9" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T9" s="75" t="s">
+        <v>9</v>
+      </c>
+      <c r="U9" s="75">
+        <v>1.4270000000000001E-3</v>
+      </c>
+      <c r="V9" s="75" t="s">
+        <v>864</v>
+      </c>
+      <c r="W9" s="75" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" ht="17">
       <c r="A10" t="s">
         <v>53</v>
       </c>
@@ -47834,8 +49874,23 @@
       <c r="Q10" s="9" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" ht="17">
+      <c r="S10" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T10" s="75" t="s">
+        <v>10</v>
+      </c>
+      <c r="U10" s="75">
+        <v>2.3289999999999999E-3</v>
+      </c>
+      <c r="V10" s="75" t="s">
+        <v>866</v>
+      </c>
+      <c r="W10" s="75" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" ht="17">
       <c r="A11" t="s">
         <v>53</v>
       </c>
@@ -47888,8 +49943,23 @@
       <c r="Q11" s="9" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" ht="17">
+      <c r="S11" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T11" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="U11" s="75">
+        <v>3.6510000000000002E-3</v>
+      </c>
+      <c r="V11" s="75" t="s">
+        <v>868</v>
+      </c>
+      <c r="W11" s="75" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" ht="17">
       <c r="A12" t="s">
         <v>53</v>
       </c>
@@ -47942,8 +50012,23 @@
       <c r="Q12" s="9" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" ht="17">
+      <c r="S12" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T12" s="75" t="s">
+        <v>12</v>
+      </c>
+      <c r="U12" s="75">
+        <v>5.6540000000000002E-3</v>
+      </c>
+      <c r="V12" s="75" t="s">
+        <v>870</v>
+      </c>
+      <c r="W12" s="75" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" ht="17">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -47996,8 +50081,23 @@
       <c r="Q13" s="9" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" ht="17">
+      <c r="S13" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T13" s="75" t="s">
+        <v>13</v>
+      </c>
+      <c r="U13" s="75">
+        <v>8.9589999999999999E-3</v>
+      </c>
+      <c r="V13" s="75" t="s">
+        <v>872</v>
+      </c>
+      <c r="W13" s="75" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" ht="17">
       <c r="A14" t="s">
         <v>53</v>
       </c>
@@ -48050,8 +50150,23 @@
       <c r="Q14" s="9" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" ht="17">
+      <c r="S14" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T14" s="75" t="s">
+        <v>14</v>
+      </c>
+      <c r="U14" s="75">
+        <v>1.3701E-2</v>
+      </c>
+      <c r="V14" s="75" t="s">
+        <v>874</v>
+      </c>
+      <c r="W14" s="75" t="s">
+        <v>875</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" ht="17">
       <c r="A15" t="s">
         <v>53</v>
       </c>
@@ -48104,8 +50219,23 @@
       <c r="Q15" s="9" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" ht="17">
+      <c r="S15" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T15" s="75" t="s">
+        <v>15</v>
+      </c>
+      <c r="U15" s="75">
+        <v>2.1679E-2</v>
+      </c>
+      <c r="V15" s="75" t="s">
+        <v>876</v>
+      </c>
+      <c r="W15" s="75" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" ht="17">
       <c r="A16" t="s">
         <v>53</v>
       </c>
@@ -48158,8 +50288,23 @@
       <c r="Q16" s="9" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" ht="17">
+      <c r="S16" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T16" s="75" t="s">
+        <v>16</v>
+      </c>
+      <c r="U16" s="75">
+        <v>3.7803000000000003E-2</v>
+      </c>
+      <c r="V16" s="75" t="s">
+        <v>878</v>
+      </c>
+      <c r="W16" s="75" t="s">
+        <v>879</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" ht="17">
       <c r="A17" t="s">
         <v>53</v>
       </c>
@@ -48212,8 +50357,23 @@
       <c r="Q17" s="3" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" ht="17">
+      <c r="S17" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T17" s="75" t="s">
+        <v>17</v>
+      </c>
+      <c r="U17" s="75">
+        <v>6.8361000000000005E-2</v>
+      </c>
+      <c r="V17" s="75" t="s">
+        <v>880</v>
+      </c>
+      <c r="W17" s="75" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" ht="17">
       <c r="A18" t="s">
         <v>53</v>
       </c>
@@ -48266,8 +50426,23 @@
       <c r="Q18" s="9" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" ht="17">
+      <c r="S18" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T18" s="75" t="s">
+        <v>18</v>
+      </c>
+      <c r="U18" s="75">
+        <v>0.11822299999999999</v>
+      </c>
+      <c r="V18" s="75" t="s">
+        <v>882</v>
+      </c>
+      <c r="W18" s="75" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" ht="17">
       <c r="A19" t="s">
         <v>53</v>
       </c>
@@ -48320,8 +50495,23 @@
       <c r="Q19" s="9" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" ht="17">
+      <c r="S19" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T19" s="75" t="s">
+        <v>19</v>
+      </c>
+      <c r="U19" s="75">
+        <v>0.19481599999999999</v>
+      </c>
+      <c r="V19" s="75" t="s">
+        <v>884</v>
+      </c>
+      <c r="W19" s="75" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" ht="17">
       <c r="A20" t="s">
         <v>53</v>
       </c>
@@ -48374,8 +50564,23 @@
       <c r="Q20" s="9" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" ht="17">
+      <c r="S20" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T20" s="75" t="s">
+        <v>20</v>
+      </c>
+      <c r="U20" s="75">
+        <v>0.29444999999999999</v>
+      </c>
+      <c r="V20" s="75" t="s">
+        <v>886</v>
+      </c>
+      <c r="W20" s="75" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" ht="17">
       <c r="A21" t="s">
         <v>53</v>
       </c>
@@ -48428,8 +50633,23 @@
       <c r="Q21" s="9" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" ht="17">
+      <c r="S21" s="74" t="s">
+        <v>53</v>
+      </c>
+      <c r="T21" s="75" t="s">
+        <v>54</v>
+      </c>
+      <c r="U21" s="75">
+        <v>0.41848000000000002</v>
+      </c>
+      <c r="V21" s="75" t="s">
+        <v>888</v>
+      </c>
+      <c r="W21" s="75" t="s">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" ht="17">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -48482,8 +50702,13 @@
       <c r="Q22" s="9" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" ht="17">
+      <c r="S22" s="76"/>
+      <c r="T22" s="76"/>
+      <c r="U22" s="76"/>
+      <c r="V22" s="76"/>
+      <c r="W22" s="76"/>
+    </row>
+    <row r="23" spans="1:23" ht="17">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -48536,8 +50761,13 @@
       <c r="Q23" s="9" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" ht="17">
+      <c r="S23" s="76"/>
+      <c r="T23" s="76"/>
+      <c r="U23" s="76"/>
+      <c r="V23" s="76"/>
+      <c r="W23" s="76"/>
+    </row>
+    <row r="24" spans="1:23" ht="17">
       <c r="A24" t="s">
         <v>53</v>
       </c>
@@ -48590,8 +50820,17 @@
       <c r="Q24" s="9" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" ht="17">
+      <c r="S24" s="74" t="s">
+        <v>890</v>
+      </c>
+      <c r="T24" s="75">
+        <v>4</v>
+      </c>
+      <c r="U24" s="76"/>
+      <c r="V24" s="76"/>
+      <c r="W24" s="76"/>
+    </row>
+    <row r="25" spans="1:23" ht="17">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -48645,7 +50884,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="17">
+    <row r="26" spans="1:23" ht="17">
       <c r="A26" t="s">
         <v>53</v>
       </c>
@@ -48687,7 +50926,7 @@
       </c>
       <c r="P26" s="10"/>
     </row>
-    <row r="27" spans="1:17" ht="17">
+    <row r="27" spans="1:23" ht="17">
       <c r="A27" t="s">
         <v>53</v>
       </c>

</xml_diff>